<commit_message>
exp: finished the code, ready to write
</commit_message>
<xml_diff>
--- a/export/tables/Table1_DescriptiveStats.xlsx
+++ b/export/tables/Table1_DescriptiveStats.xlsx
@@ -461,7 +461,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>match competitiveness</t>
+          <t>Competitiveness — Relatedness (M1)</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -492,7 +492,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>match stakeholder cocreation</t>
+          <t>Stakeholder Co-creation — Relatedness (M1)</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -523,7 +523,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>match business portfolio</t>
+          <t>Business Portfolio — Relatedness (M1)</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -554,7 +554,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>match intellectual capital</t>
+          <t>Intellectual Capital — Relatedness (M1)</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -585,7 +585,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>match digital transformation</t>
+          <t>Digital Transformation — Relatedness (M1)</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -616,7 +616,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>match financial metrics</t>
+          <t>Financial Metrics — Relatedness (M1)</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>match corporate value</t>
+          <t>Corporate Value — Relatedness (M1)</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -678,7 +678,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>tend competitiveness pos mean</t>
+          <t>Competitiveness — Positive Mean (M3)</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -709,7 +709,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>tend stakeholder cocreation pos mean</t>
+          <t>Stakeholder Co-creation — Positive Mean (M3)</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -740,7 +740,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>tend business portfolio pos mean</t>
+          <t>Business Portfolio — Positive Mean (M3)</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -771,7 +771,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>tend intellectual capital pos mean</t>
+          <t>Intellectual Capital — Positive Mean (M3)</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -802,7 +802,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>tend digital transformation pos mean</t>
+          <t>Digital Transformation — Positive Mean (M3)</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -833,7 +833,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>tend financial metrics pos mean</t>
+          <t>Financial Metrics — Positive Mean (M3)</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -864,7 +864,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>tend corporate value pos mean</t>
+          <t>Corporate Value — Positive Mean (M3)</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -895,7 +895,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>tend competitiveness neg mean</t>
+          <t>Competitiveness — Negative Mean (M3)</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -926,7 +926,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>tend stakeholder cocreation neg mean</t>
+          <t>Stakeholder Co-creation — Negative Mean (M3)</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -957,7 +957,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>tend business portfolio neg mean</t>
+          <t>Business Portfolio — Negative Mean (M3)</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -988,7 +988,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>tend intellectual capital neg mean</t>
+          <t>Intellectual Capital — Negative Mean (M3)</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1019,7 +1019,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>tend digital transformation neg mean</t>
+          <t>Digital Transformation — Negative Mean (M3)</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1050,7 +1050,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>tend financial metrics neg mean</t>
+          <t>Financial Metrics — Negative Mean (M3)</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1081,7 +1081,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>tend corporate value neg mean</t>
+          <t>Corporate Value — Negative Mean (M3)</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1112,7 +1112,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>sentiment mean</t>
+          <t>Overall ESG Sentiment</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1143,7 +1143,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>log mc</t>
+          <t>Log Market Cap</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1174,7 +1174,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>dlog mc</t>
+          <t>ΔLog Market Cap (YoY)</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1205,7 +1205,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>roa pct</t>
+          <t>ROA (%)</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1236,7 +1236,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ltdebt assets pct</t>
+          <t>LT Debt / Assets (%)</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1267,40 +1267,38 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>rnd share pct</t>
+          <t>R&amp;D / Revenue (%)</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>13226</v>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr"/>
+        <v>13196</v>
+      </c>
+      <c r="C28" t="n">
+        <v>174.9942</v>
+      </c>
+      <c r="D28" t="n">
+        <v>10207.2294</v>
+      </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>0.4055</v>
+        <v>0.4043</v>
       </c>
       <c r="G28" t="n">
-        <v>1.3882</v>
+        <v>1.382</v>
       </c>
       <c r="H28" t="n">
-        <v>3.5432</v>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+        <v>3.5241</v>
+      </c>
+      <c r="I28" t="n">
+        <v>1077161.1111</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ibes rec mean</t>
+          <t>IBES Recommendation (Mean)</t>
         </is>
       </c>
       <c r="B29" t="n">

</xml_diff>